<commit_message>
Update: Set 1-strike prune rule and improve db consistency
</commit_message>
<xml_diff>
--- a/注册结果.xlsx
+++ b/注册结果.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2008,6 +2008,3838 @@
       </c>
       <c r="J41" t="inlineStr"/>
     </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>xipCloud</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://xipcloudy.com/zh</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>gridley62efcd@yr.accesswiki.net</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>CordCloud</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://www.cordc.net/</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>jesse62efd8@5e.tohal.org</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>FnF 机场</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://fnff.top/manyvoices/zh</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>抖云加速</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/1656.html</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>emerick62efec@cw.accesswiki.net</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>大哥云</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://aff02.dgy02.com/#/register?code=TdJ9zhmt</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>rosabel62f01b@ua.cloudvxz.com</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>云图小镇</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://20260223.dev.tarolink.top/auth/register?code=H6q1</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>iKuuu VPN</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://ikuuu.org/auth/login</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>reviere62f02c@zu.accesswiki.net</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>赔钱机场</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://xn--mes358aby2apfg.com/#/register?code=vYU0rYqI</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>chas62f030@bb.accesswiki.net</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>大机场 Big Airport</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://xn--mesr8b36x.net/#/register?code=ZArZYgxI</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>注册失败-发验证码失败</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>请求发送验证码接口失败/被拦截</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>奈思云</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://2nss.com/#/register?code=HoWU9UzZ</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>andy62f03c@1e.shopsprint.org</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>速子云</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://get.tachban.xyz/#/register?code=ov17PIi1</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>folger62f040@4z.hush2u.com</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Sakura Cat 樱花猫</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://c2-sakuracat.com/register?code=gNQyKqqG</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>barfuss62f046@g9.shopsprint.org</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>接口返回错误: {'success': False, 'data': ''}</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Gsou Cloud</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/1065.html</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>雨燕云</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://new4.yuyan.online/#/register?code=Y91yRm56</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>https://173.249.210.26/s/b590020ef542fd01c5ac000c13ff493f</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>173.249.210.26</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>最低0元/月 250.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>雷霆</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://hi.leiting.uk/invite/jKQeDYtR</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>jojo62f05b@ed.hush2u.com</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Bridge the Wise</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/987.html</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>laverne62f061@u7h.sixthirtydance.org</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>次元云</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https://ciyy.cc/index.php#/register?code=SDy1BBg2</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>cressy62f068@0m.sixthirtydance.org</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>7速云</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://7sucloud.net/register?code=BUO5DT2C</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>killigrew62f06a@2k.shopsprint.org</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>木瓜云</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/780.html</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>次元链接</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/775.html</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>tobye62f07e@te.hush2u.com</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Paper Plane</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https://zfj.so/auth/register?code=a2d354c8d2</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>marian62f0be@08.shopsprint.org</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>need_tos</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>猫熊网络加速器</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>https://mxwljsq.com/auth/login</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>amin62f0c7@zt.shopsprint.org</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>接口返回错误: {'detail': 'Not Found'}</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>NyaCloud</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>https://xn--9kqw7o.com/</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>irene62f0cb@7u.cloudvxz.com</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Web3 加速器</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>https://web3jsq.vip/f/7209DeWk</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>V2 Network</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>https://v2cn.com/</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ninette62f0d3@qq.tohal.org</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>KyCloud</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>https://cp.cloudnx.cc/aff.php?aff=59467</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>lurline62f0da@ju.cloudvxz.com</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Xlinkworld</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/546.html</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>lindi62f0e4@f5.tohal.org</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Just My Socks</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>https://justmysocks3.net/members/</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>grath62f10b@u9.accesswiki.net</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Mie Link 羊圈机场</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>https://mielink.org/zh-TW</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>leonidas62f115@sl.accesswiki.net</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>接口返回错误: {'code': 400, 'message': '此路径必须使用加密访问'}</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>CMY Network 红莓网络</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>https://cmy3.network/</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>justinn62f11c@sf.sixthirtydance.org</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>接口返回错误: {'code': 400, 'message': '此路径必须使用加密访问'}</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>MilkCat 奶猫</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>https://catweb.jjjxgc.com/#/register?code=zX0OMoQr</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>hertzfeld62f121@ek.sixthirtydance.org</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>饿饭CC云</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>https://efanccyun.org</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>fee62f129@gk.cloudvxz.com</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>青云梯</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>https://qytcc01a.qingyunti.pro/verify?next=%2Fregister%3Faff%3DwMlUHVM0</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>sethrida62f12b@t2.sixthirtydance.org</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>TomatoCloud</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>https://tomatocloud.me/account?action=register&amp;code=Lzw71T</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>CitrusLab</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>https://h2breeze.com/register?aff=lDbdDtHB</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>忍者云</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>https://renzhe.cloud/</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>cristen62f132@wn.sixthirtydance.org</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>科技熊</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>https://kjxclub.com/auth/register?code=eerr</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>cohberg62f136@v2.tohal.org</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>https://www.yuansu.app/#/invite/TZ8BMBES</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>barber62f13c@zz.hush2u.com</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>prprCloud</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>https://prpr.96110.cn.com/</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>lorrin62f141@6y.sixthirtydance.org</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>速鹰666</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>https://sy77a12.com/auth/register?code=nEmD</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>kelcie62f145@16.sixthirtydance.org</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>桔子云</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>https://jzy66222.xyz/auth/register?code=ajJa</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>jeanelle62f149@tw.hush2u.com</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>BestVPN!</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>https://best.invitevp.com/#/register?code=oFipIA9S</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>alethea62f14e@in.tohal.org</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>GLaDOS</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>https://glados.space/</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>chloette62f152@tfh.shopsprint.org</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>WestData</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>https://wd-gold.com/aff.php?aff=1327</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>salomie62f156@vq.accesswiki.net</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr"/>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>CreamData 奶油</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>https://www.naiyovpn.com/?aff=20#signup</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>kaia62f158@9s.shopsprint.org</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr"/>
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>泡芙云</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>https://x.paofu.io/WAF/VERIFY/CAPTCHA?info=XjGx1hLlunoF7bP5QpZH%2FxKA6pqsc6jX1zRVkgw4UQhtbdsSWhMWtxwtW%2BOrKP5F1YxiEYTUFw2mrsKbuaDWLz2eZNYlahG%2B8KYSj4YARxTTspg1dWFNJHYy&amp;from=%2Fregister%3Fcode%3DJ72lqgFj</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>s8g33zwbvt@deltajohnsons.com</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr"/>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>瑶瑶领先</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>https://yyssr.org/auth/register?code=a7ad7c24bb</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>fltknkppsd@deltajohnsons.com</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>need_tos</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Boslife</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>https://www.blnew.com/#/register?code=NlciSgn2</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>tfv6x2o88m@deltajohnsons.com</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>纷达网络</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>https://fenda.cloud/auth/login</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>注册失败-发验证码失败</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>g7axc7zkdz@deltajohnsons.com</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>请求发送验证码接口失败/被拦截</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Fastlink</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>https://a12.flaffa03.cc/verify?next=%2Fauth%2Fregister%3Fcode%3DhRfC</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>4dcp940vn5@bwmyga.com</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr"/>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>涩龙云</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>https://www.selom.xyz/#/register?code=LLQNKXcA</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>https://orange.slsub.com/subs/0b31774f5625c6043847ec7b0168d5dd</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>orange.slsub.com</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr"/>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>最低0元/月 1024.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Nerwo 机场</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>https://share.eleven.observer/auth/register.html?code=bvvf</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>我们所向往的 wmsxwd</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>https://wmsxwd-3.men/#/register?code=4Qa6zQxl</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>sibley62f195@64l.shopsprint.org</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>AmyTelecom</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>https://www.amytele.co/aff.php?aff=17</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>elisabet62f19a@29.accesswiki.net</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>魅影极速</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>https://www.myjs.net/</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>zippel62f19d@o8.cloudvxz.com</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>X-Air</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>https://my.x-air.app:666/#/register?aff=34041</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>stander62f1a3@4u.tohal.org</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Bitz Net</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>https://dash.gobitz.net/#/register?code=cNQOuMNq</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>接口返回错误: {'message': 'The GET method is not supported for t</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Ayanami！（色色小站）</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>https://www.sesexiaozhan.com/#/register?code=Xq8mcGFd</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>terryl62f1a9@mt.tohal.org</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Coffee Cloud</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>https://xn--9kqp0mora.com/#/register?code=s5MEj7Ro</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>latea62f1ab@lt.shopsprint.org</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr"/>
+      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>奈云</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>https://aff.v2ny.mom?path=register&amp;code=T86GRpsu</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>dunseath62f1b0@x3f.shopsprint.org</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr"/>
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>一枝红杏</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>https://order.yizhihongxing.club</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>tremayne62f1b8@yt.cloudvxz.com</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr"/>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>BFG 加速</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>https://www.bfgok.com/auth/register?code=GQDdMl</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>alexia62f1c0@tuj.accesswiki.net</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr"/>
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Godetia</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>https://lkjhl.goodoetoioa.xyz/#/register?code=oj7lAyEn</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>https://dsfhi.dwhufe.bar/s/2d5c8da72835d9fa72726c86356a667b</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>dsfhi.dwhufe.bar</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr"/>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>最低29.4元/月 85.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>白月光机场</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>https://www.sibker.com/register?invite_code=MLRoveBn</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>devinne62f1cf@ew.cloudvxz.com</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr"/>
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Infini Port</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>https://console.infiniport.xyz/#/register?code=cd00IGfe</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>waldon62f1d5@u7h.sixthirtydance.org</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Paoluz 跑路云</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>https://paoluz.link/auth/register?code=gZNc</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>karil62f1d7@6c.tohal.org</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr"/>
+      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>SaySS</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>https://www.sayss.net/#/register</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr"/>
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>飞数机场</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/102.html</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>chane62f1dd@9c.cloudvxz.com</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr"/>
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Gatern 机场</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>https://s.gtoyes.com/index.php/store/ding-yue-fu-wu</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>shinberg62f1e4@77.cloudvxz.com</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>SpeedCAT 闪电猫</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>https://scvbaff-hezb07.cc/verify?next=%2Fauth%2Fregister%3Fcode%3DDwPz</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>berlyn62f1ed@sw.accesswiki.net</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Anyland</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>https://anyland.xyz/#/register?code=PHOMVrCA</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>annissa62f1f2@d5j.accesswiki.net</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr"/>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>GTK PW</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>https://board.gtk.pw/#/register?code=PoPXZgzj</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr"/>
+      <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr"/>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>最低0元/月 100.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>FlyingBird 飞鸟机场</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>https://fba01.fbva-hen.cc/auth/register?code=DLmG</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>berglund62f1fc@ry.cloudvxz.com</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>ENET 机场</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>https://www.easyenable.com/#/register?code=Ikvt9dR8</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>CATNET 机场</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>https://0703.catnet01-c6ti90mq.top/#/register?code=yqbRbGui</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>feodora62f202@hd.accesswiki.net</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>鹿语云</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/1859.html</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>roana62f208@yu.shopsprint.org</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr"/>
+      <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>悠兔机场</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>https://youtunice.com?path=register&amp;code=Di40kVJz</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>cha62f24a@y3.cloudvxz.com</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr"/>
+      <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>扬帆云</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>https://yawtt.net/register?code=iMKVpg72</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>natassia62f24d@mx.shopsprint.org</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Cyber Guard</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>https://cyberguard.best/#/register?code=ILTQCdgz</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>aleen62f252@ch.shopsprint.org</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr"/>
+      <c r="H120" t="inlineStr"/>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>肥猫云</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>https://fcvipaffa05.cc/login#/register?code=QmcPwI0U</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr"/>
+      <c r="H121" t="inlineStr"/>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>YkkCloud</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>https://panel.ykkk.best/#/register?code=atY9N92D</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>farmann62f262@zg.cloudvxz.com</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr"/>
+      <c r="H122" t="inlineStr"/>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>飞天猪</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>http://a09.ftzvipaffa02.cc/verify?next=%2F#/register?code=ltSl4YJR</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr"/>
+      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr"/>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>最低7.0元/月 50.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Boost Net</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>https://boostqz.com/?path=register&amp;code=9cw25cQ8</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>zina62f269@1b.sixthirtydance.org</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr"/>
+      <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>接口返回错误: {'error': {'code': '404', 'message': 'The page cou</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Dragonfly 蜻蜓</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>https://9dragonfly.com/register?affiliate=RK-eAQ7u3Q</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>paulita62f26b@yi.sixthirtydance.org</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>E-IX 机场</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>https://ap.cdn.e-ix.com/#/register?code=IJVP9uMc</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr"/>
+      <c r="H126" t="inlineStr"/>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>接口返回错误: {'message': '邮箱验证码有误'}</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>AnyNet</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>https://anynet.me/#/register?code=FpMYlLD5</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>txnz6vb879@deltajohnsons.com</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr"/>
+      <c r="H127" t="inlineStr"/>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>WaveNebula 电波星云</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>https://user.fk8w.com/#/register?code=7tMWDl1w</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>zia0ww9v2c@deltajohnsons.com</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr"/>
+      <c r="H128" t="inlineStr"/>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>蓝莓速递</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>https://berryexpress.top/#/register?code=TB3mbSpM</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>注册失败-邮箱不支持</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>yjr4wzeyka@deltajohnsons.com</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr"/>
+      <c r="H129" t="inlineStr"/>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>所有备用邮箱均被该站点拒绝</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>地鼠机场</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>https://nbvpn.top/#/register?code=3wUFtGx6</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>regqh5ldyjl@maildrop.cc</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr"/>
+      <c r="H130" t="inlineStr"/>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>省钱机场</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>https://xn--mes358ag1lu22a.com/#/register?code=AOXcP4Ph</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>reg81o7d9kk@maildrop.cc</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr"/>
+      <c r="H131" t="inlineStr"/>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>维度云</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>https://weidu.io/#/auth?invite=uuxWk79E</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>regzrgqmwyj@maildrop.cc</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr"/>
+      <c r="H132" t="inlineStr"/>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>V2ge</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>https://a.v2ge.me/#/register?code=vg2hcSWq</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>https://ttt-fhdcaqbigu.cn-shenzhen.fcapp.run/s/a2d56efc40a974bca6d68a40ae55a63c</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>ttt-fhdcaqbigu.cn-shenzhen.fcapp.run</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr"/>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>最低0元/月 100.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Nachoneko</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>https://nachoneko.cc/#/register?code=DPdIrBsC</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>reg6f75kq7d@maildrop.cc</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr"/>
+      <c r="H134" t="inlineStr"/>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>茶艺云</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>https://cloud.teaartcloud.com/#/register?code=RV6xMOtm</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>regl4q30fkv@maildrop.cc</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr"/>
+      <c r="H135" t="inlineStr"/>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>接口返回错误: {'message': 'The route api/v1/api/v1/passport/auth</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>滕王阁机场</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>https://twg520.com/#/register?code=qfrq9M25</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>regq7siysen@maildrop.cc</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr"/>
+      <c r="H136" t="inlineStr"/>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Danke Cloud</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>https://a10.danke.sbs/#/register?code=rLnJD5a2</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>bibbye62f2be@cc.sixthirtydance.org</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr"/>
+      <c r="H137" t="inlineStr"/>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>凌速加速器 / LingSpeed</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/4550.html</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>angie62f2ca@le.accesswiki.net</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr"/>
+      <c r="H138" t="inlineStr"/>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>FlyBit</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>https://goflybit.com#/register?code=78E34u9V</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>bertha62f2f1@h7.hush2u.com</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr"/>
+      <c r="H139" t="inlineStr"/>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>表哥云</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>https://biaoge.us/portal/register?code=JnaSNApe</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>halette62f2f3@9.tohal.org</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr"/>
+      <c r="H140" t="inlineStr"/>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>狮子云</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>https://dash.shizi.in/portal/register?code=DKBxnL7Q</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>deeann62f2f7@ft.hush2u.com</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr"/>
+      <c r="H141" t="inlineStr"/>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Build: Integrate jichangnodelist resources, add 5 new channels and 30+ airports
</commit_message>
<xml_diff>
--- a/注册结果.xlsx
+++ b/注册结果.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J141"/>
+  <dimension ref="A1:J191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5840,6 +5840,1962 @@
       </c>
       <c r="J141" t="inlineStr"/>
     </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>蓝莓桥</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>https://berrypass.net/#/register?code=MWJc9hyM</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>注册失败-邮箱不支持</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>noni62f2fd@6t.tohal.org</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr"/>
+      <c r="H142" t="inlineStr"/>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>所有备用邮箱均被该站点拒绝</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>迅达 VPN</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>https://sulianproxy.com/register?code=qRRAlOD9</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>087xwx7a50@mailpwr.com</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr"/>
+      <c r="H143" t="inlineStr"/>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>团子猫通信</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>https://dash.tuanzimao.net/#/register?code=9hxIbhfl</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>https://sub-tuanzimao.260311.xyz/s/50efc9866850430e72832896325c4524</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>sub-tuanzimao.260311.xyz</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr"/>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>最低4.83元/月 50.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Neko Cloud</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>https://my.nekocloud.top/#/register?code=T37z4XoD</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>dyhiw0masam2@picomail.biz</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr"/>
+      <c r="H145" t="inlineStr"/>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>接口返回错误: {'message': 'The route api/v1/api/v1/passport/auth</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Phantom</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>https://pin.dianping.men/auth/register?code=KjGTJNgb</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>wmedwygao@emlpro.com</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr"/>
+      <c r="H146" t="inlineStr"/>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>SSONE</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>https://hello-ssone.com/register?aff=3Ypczm9L</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>vypimigik1m3@picomail.biz</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr"/>
+      <c r="H147" t="inlineStr"/>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>星币机场</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/4382.html</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>jrpjdmkfn@emlhub.com</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr"/>
+      <c r="H148" t="inlineStr"/>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>ToDesk</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>https://todesk.io/auth/register?affid=156884</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>levypekymow3@10mail.info</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr"/>
+      <c r="H149" t="inlineStr"/>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>千速云</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>https://www.1000ws.top/#/register?code=gpBSiKhr</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>bysamuf0hab2@mailtowin.com</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr"/>
+      <c r="H150" t="inlineStr"/>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>接口返回错误: {'detail': 'Method Not Allowed'}</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>念云</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>https://xnyun.wiki/</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>mrrxnzgao@emlpro.com</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr"/>
+      <c r="H151" t="inlineStr"/>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>LiZiOne</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>https://lizione.com/#/register?code=voKSUQaR</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr"/>
+      <c r="H152" t="inlineStr"/>
+      <c r="I152" t="inlineStr"/>
+      <c r="J152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>oixCloud</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>https://oixcloud.com/auth/register?affid=156884</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>gohyw1n0z1j3@maximail.fyi</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr"/>
+      <c r="H153" t="inlineStr"/>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>特朗普云</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>https://trumpyun.com/index.php/#/register?code=odAPxA2O</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>注册成功</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>https://api1.trumpyun1.com/s/da4da2d674e1ed7cc55dea5b60b8a8e8</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>api1.trumpyun1.com</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr"/>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>最低0元/月 300.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>隐云</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>https://wkacc.xyz/?code=a7e5fbff</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>hep0lyb0sih2@pickmail.org</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr"/>
+      <c r="H155" t="inlineStr"/>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Global Cloud 全球云</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>https://gc01.globalyun.cc/</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr"/>
+      <c r="H156" t="inlineStr"/>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>飞猫云</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>https://vip02.flyingcat.work/</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr"/>
+      <c r="H157" t="inlineStr"/>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>StarTrail 星轨</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>https://plinkc.sbs/#/register?code=XXYXJzO8</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>pybagosigyb3@pickmemail.com</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr"/>
+      <c r="H158" t="inlineStr"/>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>158</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>eueu</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>https://eueua.cc/#/register?code=oiTWeLYk</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>akabqhthaoclsx@dropmail.me</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr"/>
+      <c r="H159" t="inlineStr"/>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>159</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>光年梯</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>https://vpnbaycom.gntvipaff.cc/#/?code=YgPQcmp2</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>akabqiondmhdjy@dropmail.me</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr"/>
+      <c r="H160" t="inlineStr"/>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>160</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>YoYoo</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>https://yoyoo.net/#/register?code=FdNcky8y</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>http://152.136.168.107:81/s/f375a079b52473d2c002f4f44b4a3a89</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>152.136.168.107:81</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr"/>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>最低0元/月 2.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>161</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>神龙机场</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>https://shenlong123.cc/#/register?code=5M5JyNMs</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>zutyminafom0w2@10mail.xyz</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr"/>
+      <c r="H162" t="inlineStr"/>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>162</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>HK-BEUP</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>https://www.beupisp.com/register?code=OKUf5v4p</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>gof0w0hewew3@mailtowin.com</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr"/>
+      <c r="H163" t="inlineStr"/>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>163</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>墨菲云</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>https://portal.mofeiyun.com/#/register?code=bTZNKGeX</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>fivuwyjikel3@picomail.biz</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr"/>
+      <c r="H164" t="inlineStr"/>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>164</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>One Step</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>https://login.onestep.lat/#/register?code=K0awGg26</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr"/>
+      <c r="H165" t="inlineStr"/>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>165</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>PyroCloud</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>https://pyrocloud.xyz/#/auth?invite=uu43Srnu</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>alpnzqaau@10mail.org</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr"/>
+      <c r="H166" t="inlineStr"/>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>166</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>悠云 UOCloud</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>https://www.uoyun.com/#/register?code=pbfcvTZl</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>m1m1tom0lug3@picomail.biz</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr"/>
+      <c r="H167" t="inlineStr"/>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>167</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>咩咩速联</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>https://eck8.miemie.uk/#/register?code=OvKgtCps</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>xhhbajzho@emltmp.com</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr"/>
+      <c r="H168" t="inlineStr"/>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>168</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Tomato 番茄🍅</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>https://tmt.lat</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr"/>
+      <c r="H169" t="inlineStr"/>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>169</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>TAPCloud</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>https://tapcloud.me/web/#/login?code=tRY553xG</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr"/>
+      <c r="H170" t="inlineStr"/>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>170</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>SingLink 星连</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>https://mysinglinkweb.com/en#/register?code=PiJ4wqka</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>注册成功</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>veg1beh1j1t3@pickmemail.com</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr"/>
+      <c r="H171" t="inlineStr"/>
+      <c r="I171" t="inlineStr"/>
+      <c r="J171" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>171</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>鱼云机场</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>https://yuwan.xyz/register?code=1k1ueRng</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>yrvdlahao@emlpro.com</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr"/>
+      <c r="H172" t="inlineStr"/>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">接口返回错误: {'error': {'code': '403', 'message': 'Forbidden', </t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>172</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>唯兔云</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>https://vip01.onlyrabbit.cc/#/?code=ZdDzdK8Q</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>akbffjuif@yomail.info</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr"/>
+      <c r="H173" t="inlineStr"/>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>173</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>星岛梦</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>https://vpnbay01.xdmvipaff.cc/#/?code=b5iohwDN</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>f1tolum0l1m2@maximail.fyi</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr"/>
+      <c r="H174" t="inlineStr"/>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>174</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>光速云</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>https://gsy01.lightspeed.club/</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr"/>
+      <c r="H175" t="inlineStr"/>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>175</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>NMY 牛马云</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>https://board.nmy.skin/#/register?code=e5tdJF28</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>https://media.wyidc.xyz/s/907fa3507fdc44c0cffba17af08e3648</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>media.wyidc.xyz</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr"/>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>最低1.0元/月 50.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>176</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Matcha Network</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>https://matcha.su/#/register?code=AKTUJuX2</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>zmspvnkfn@emlhub.com</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr"/>
+      <c r="H177" t="inlineStr"/>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>177</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>极连云</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>https://vpnbay01.jlcvipaff.cc#/register?code=x7YajRfc</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>09g2aq08a4@freeml.net</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr"/>
+      <c r="H178" t="inlineStr"/>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>178</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>寿司云VPN</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/3566.html</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>hol0lew0nik2@mail2me.co</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr"/>
+      <c r="H179" t="inlineStr"/>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>179</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>SkyCloud</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>https://panel.skycloud.lol/zh/auth/signup?referrer=FYG1DtiU</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>https://board.skycloud.lol/s/407ec5165a6f5e2fc213777b882e1d75</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>board.skycloud.lol</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr"/>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>最低0元/月 25.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>180</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>CrossWall</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>https://www.crosswall.org/#/register?code=eHZ1cb6d</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>http://162.19.79.201/s/06bdf1bc09acf1dc506d6db22574eb8d</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>162.19.79.201</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr"/>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>最低0元/月 500.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>181</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>咕噜咕噜</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>https://gl-ez.pages.dev/#/register?code=jLBit6Uh</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>qywhdokfn@emlhub.com</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr"/>
+      <c r="H182" t="inlineStr"/>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>182</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>美乐云</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>https://www.v3ml.com#/register?code=eur0SOGQ</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>https://2027.v3ml.cc/s/10212e0bdca01426ce20421dceef7894</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>2027.v3ml.cc</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr"/>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>最低0元/月 128.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>183</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>山海云</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>https://shanhai.cfd/#/register?code=GRARlFsr</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>z1f0fikizab3@maximail.fyi</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr"/>
+      <c r="H184" t="inlineStr"/>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>184</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>奶茶机场</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>https://naichachong.com/#/register?code=3IS2GFHP</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>fipisefepunan2@10mail.xyz</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr"/>
+      <c r="H185" t="inlineStr"/>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>185</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>酷酷云 KuKuYun</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>https://a09.kkyvipaff02.cc/register?aff=hboaGlNk</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr"/>
+      <c r="H186" t="inlineStr"/>
+      <c r="I186" t="inlineStr"/>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>最低12.0元/月 100.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>186</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>KooDog</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>https://www.kdcloud.uk/#/register?code=oMrF1orI</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>注册失败-发验证码失败</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr"/>
+      <c r="H187" t="inlineStr"/>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>请求发送验证码接口失败/被拦截</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr"/>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>187</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Flywarp 飞梭机场</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>https://79fac683dfd5d99a.fs01.cc/#/register?code=YVYMBKL4</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>注册成功</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>henog1dilefeb4@10mail.xyz</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>https://9gma2kfq.hhkk123.asia/f7m2x9qz/f0b916a8b1295e325e126b6538e68969</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>9gma2kfq.hhkk123.asia</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr"/>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>最低0元/月 100.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>188</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>鱼鱼的超级机场</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>https://288811.xyz/#/register?code=kEx2akw2</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>注册失败-收不到验证码</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>vyjevinaj1m2@mail2me.co</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr"/>
+      <c r="H189" t="inlineStr"/>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>临时邮箱/Gmail均未收到验证码</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr"/>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>189</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>OMOT</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/3229.html</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr"/>
+      <c r="H190" t="inlineStr"/>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr"/>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>190</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Perfect Link</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>https://www.perlnk.com/#/auth?invite=uUn8UTh3</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>myzegoj1p1nif4@10mail.xyz</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr"/>
+      <c r="H191" t="inlineStr"/>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix: correct newline formatting in all_nodes.txt and add thread lock for safe writing
</commit_message>
<xml_diff>
--- a/注册结果.xlsx
+++ b/注册结果.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,7 +489,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>huesman62f5f0@u.accesswiki.net</t>
+          <t>perry62f634@t1.sixthirtydance.org</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -508,26 +508,26 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FlowerCloud 花云</t>
+          <t>Viking Links</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://api-flowercloud.com/aff.php?aff=17304</t>
+          <t>https://feeds.viking-links.tech/#/login?code=MaFTn476</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>跳过-Cloudflare</t>
+          <t>已注册-登录成功</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>carvey62f5f0@4hk.accesswiki.net</t>
+          <t>moneyflysubssr@gmail.com</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -535,56 +535,18 @@
           <t>Sikeming001@</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Cloudflare 防护</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Viking Links</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>https://feeds.viking-links.tech/#/login?code=MaFTn476</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>已注册-登录成功</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>moneyflysubssr@gmail.com</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Sikeming001@</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>https://pics9.sknil-gnikiv.com/wx5TqEUTwXks/v1/w7LQhnaSTnjD/VikingLinks?token=748dcb17331d3175ffab97ae65b2e4b4.723v29gnu18.jpg</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://pics9.sknil-gnikiv.com/wx5TqEUTwXks/v1/w7LQhnaSTnjD/VikingLinks?token=748dcb17331d3175ffab97ae65b2e4b4.7553ahov29g.jpg</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>pics9.sknil-gnikiv.com</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr">
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
         <is>
           <t>最低27.5元/月 250.0GB</t>
         </is>

</xml_diff>

<commit_message>
Enhance: Multi-format subscription parsing (YAML/Clash support) and URI reverse generation
</commit_message>
<xml_diff>
--- a/注册结果.xlsx
+++ b/注册结果.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J261"/>
+  <dimension ref="A1:J381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10456,6 +10456,4558 @@
       </c>
       <c r="J261" t="inlineStr"/>
     </row>
+    <row r="262">
+      <c r="A262" t="n">
+        <v>261</v>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Bocchi</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>https://xb.bocchi.ooo/#/register?code=4skRa5AQ</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr"/>
+      <c r="H262" t="inlineStr"/>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J262" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>262</v>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>SsdAirport</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>https://bangpi.top?path=register&amp;code=p1HsQa0W</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr"/>
+      <c r="H263" t="inlineStr"/>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J263" t="inlineStr"/>
+    </row>
+    <row r="264">
+      <c r="A264" t="n">
+        <v>263</v>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>万达云</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>https://app.wdycenter.com/register?code=mfnTlrSw</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr"/>
+      <c r="H264" t="inlineStr"/>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J264" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" t="n">
+        <v>264</v>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>柚子兔网络</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>https://yzt.moe/#/register?code=ktDtwtiD</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr"/>
+      <c r="H265" t="inlineStr"/>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J265" t="inlineStr"/>
+    </row>
+    <row r="266">
+      <c r="A266" t="n">
+        <v>265</v>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>五树云</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>https://xiaomiaff.pro/register.html?invitecode=8UctYVq0</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr"/>
+      <c r="H266" t="inlineStr"/>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J266" t="inlineStr"/>
+    </row>
+    <row r="267">
+      <c r="A267" t="n">
+        <v>266</v>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>蜂窝加速器</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>https://h.fengwo.online/#/login?code=bbAilrMO</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>注册失败-发验证码失败</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr"/>
+      <c r="H267" t="inlineStr"/>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>请求发送验证码接口失败/被拦截</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr"/>
+    </row>
+    <row r="268">
+      <c r="A268" t="n">
+        <v>267</v>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>NyanSS 喵喵云</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/1473.html</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr"/>
+      <c r="H268" t="inlineStr"/>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr"/>
+    </row>
+    <row r="269">
+      <c r="A269" t="n">
+        <v>268</v>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>PK Cloud 皮卡丘机场</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>https://pkhub.net/#/login?code=OuCU7jw4</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr"/>
+      <c r="H269" t="inlineStr"/>
+      <c r="I269" t="inlineStr"/>
+      <c r="J269" t="inlineStr"/>
+    </row>
+    <row r="270">
+      <c r="A270" t="n">
+        <v>269</v>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>尔湾云</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>https://erwan.cc/auth/register?code=Lp8Mst</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr"/>
+      <c r="H270" t="inlineStr"/>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr"/>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>270</v>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>流星 VPN</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/1420.html</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr"/>
+      <c r="H271" t="inlineStr"/>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr"/>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>271</v>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>GOHAHA</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/1416.html</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr"/>
+      <c r="H272" t="inlineStr"/>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr"/>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>272</v>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>独角兽机场</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>https://91unicorn.cloud/#/register?code=QjfbQ0DD</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr"/>
+      <c r="H273" t="inlineStr"/>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr"/>
+    </row>
+    <row r="274">
+      <c r="A274" t="n">
+        <v>273</v>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>红岸加速</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>https://hongango.vip#/register?code=6yzVxr0l</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr"/>
+      <c r="H274" t="inlineStr"/>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr"/>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>274</v>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>卡荔云</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/1393.html</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr"/>
+      <c r="H275" t="inlineStr"/>
+      <c r="I275" t="inlineStr"/>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>最低0元/月 520.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="n">
+        <v>275</v>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>小旋风机场</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>https://a04.xxfvipaff.pro/#/register?inviteCode=FFA946C92AE8</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr"/>
+      <c r="H276" t="inlineStr"/>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J276" t="inlineStr"/>
+    </row>
+    <row r="277">
+      <c r="A277" t="n">
+        <v>276</v>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>BigME 大米加速</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>https://1s.bigmeok.me/user#/register?code=WqCa8IRh</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr"/>
+      <c r="H277" t="inlineStr"/>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr"/>
+    </row>
+    <row r="278">
+      <c r="A278" t="n">
+        <v>277</v>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>淘气兔</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/1364.html</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr"/>
+      <c r="H278" t="inlineStr"/>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr"/>
+    </row>
+    <row r="279">
+      <c r="A279" t="n">
+        <v>278</v>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Arisaka</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/1360.html</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr"/>
+      <c r="H279" t="inlineStr"/>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr"/>
+    </row>
+    <row r="280">
+      <c r="A280" t="n">
+        <v>279</v>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>ikun VPN</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/1347.html</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>跳过-关闭注册</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr"/>
+      <c r="H280" t="inlineStr"/>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>站点已关闭注册</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr"/>
+    </row>
+    <row r="281">
+      <c r="A281" t="n">
+        <v>280</v>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>特价机场</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>https://82af8b68-c1c0-4897-af7e-bddf32c69b2f.75733.xyz/#/register?code=ABH5upjf</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>注册失败-发验证码失败</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr"/>
+      <c r="H281" t="inlineStr"/>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>请求发送验证码接口失败/被拦截</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr"/>
+    </row>
+    <row r="282">
+      <c r="A282" t="n">
+        <v>281</v>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>NanoCloud</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>https://edu.uodoo.bid/auth/register?code=5jhGJOZU</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr"/>
+      <c r="H282" t="inlineStr"/>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr"/>
+    </row>
+    <row r="283">
+      <c r="A283" t="n">
+        <v>282</v>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>紫鸟 VPN</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>https://ziniao.cc/#/register?code=dNNBmZsm</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr"/>
+      <c r="H283" t="inlineStr"/>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr"/>
+    </row>
+    <row r="284">
+      <c r="A284" t="n">
+        <v>283</v>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>IDCNLink</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>https://idcn.link/register?code=pQ69A2Ig</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr"/>
+      <c r="H284" t="inlineStr"/>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr"/>
+    </row>
+    <row r="285">
+      <c r="A285" t="n">
+        <v>284</v>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>跨境 Cloud</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>https://wbe-agent.kuajing.uk/auth/register?code=KF1m</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr"/>
+      <c r="H285" t="inlineStr"/>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr"/>
+    </row>
+    <row r="286">
+      <c r="A286" t="n">
+        <v>285</v>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>爬兔兔 VPN</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>https://patutu.xn--cesw6hd3s99f.com/#/register?code=wvBj813R</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr"/>
+      <c r="H286" t="inlineStr"/>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>接口返回错误: {'status': 'fail', 'message': '邮箱验证码有误', 'data': N</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr"/>
+    </row>
+    <row r="287">
+      <c r="A287" t="n">
+        <v>286</v>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>火烧云</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>https://hsy88.org/#/register?code=CojtEDjG</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr"/>
+      <c r="H287" t="inlineStr"/>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr"/>
+    </row>
+    <row r="288">
+      <c r="A288" t="n">
+        <v>287</v>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>穿云箭</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>https://rocket123.uk/#/register?code=TVvV95xA</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr"/>
+      <c r="H288" t="inlineStr"/>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr"/>
+    </row>
+    <row r="289">
+      <c r="A289" t="n">
+        <v>288</v>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>扑克云</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>https://panel.pokeryun.top/zh/#/auth/signup;referral=9o4la3T2</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr"/>
+      <c r="H289" t="inlineStr"/>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr"/>
+    </row>
+    <row r="290">
+      <c r="A290" t="n">
+        <v>289</v>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>大讯云</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>https://daxun.xyz/#/register?code=AVLIiiEd</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr"/>
+      <c r="H290" t="inlineStr"/>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>接口返回错误: {'message': ''}</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr"/>
+    </row>
+    <row r="291">
+      <c r="A291" t="n">
+        <v>290</v>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>云兔</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>https://yuntu.pro/#/register?code=k4KtoNXi</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr"/>
+      <c r="H291" t="inlineStr"/>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr"/>
+    </row>
+    <row r="292">
+      <c r="A292" t="n">
+        <v>291</v>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Poless VPN</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>https://v.diless.com/#/register?code=lXBqDb7s</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr"/>
+      <c r="H292" t="inlineStr"/>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr"/>
+    </row>
+    <row r="293">
+      <c r="A293" t="n">
+        <v>292</v>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>三番云</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>https://3fancloud.net/#/register?code=nYOQmF8l</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr"/>
+      <c r="H293" t="inlineStr"/>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr"/>
+    </row>
+    <row r="294">
+      <c r="A294" t="n">
+        <v>293</v>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>极速云</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>https://w1.jisucloudow.com:8888#/register?code=VW1a82Ds</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr"/>
+      <c r="H294" t="inlineStr"/>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t xml:space="preserve">接口返回错误: </t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr"/>
+    </row>
+    <row r="295">
+      <c r="A295" t="n">
+        <v>294</v>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>TNT Cloud</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>https://a05.tntvipaffb08.cc/#/register?code=zwGrC8KX</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr"/>
+      <c r="H295" t="inlineStr"/>
+      <c r="I295" t="inlineStr"/>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>最低8.17元/月 60.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="n">
+        <v>295</v>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Lray</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>https://lray.dlgisea.com/#/login?code=AcD5xfrX</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr"/>
+      <c r="H296" t="inlineStr"/>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr"/>
+    </row>
+    <row r="297">
+      <c r="A297" t="n">
+        <v>296</v>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>银河云</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>https://webcc01.galaxycloud.pro/login#/register?code=cogo468J</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>注册成功</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr"/>
+      <c r="H297" t="inlineStr"/>
+      <c r="I297" t="inlineStr"/>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>最低0元/月 1000.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="n">
+        <v>297</v>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Fancy Network</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>https://dash.justfancy.net/register?code=RGIksNCT</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr"/>
+      <c r="H298" t="inlineStr"/>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr"/>
+    </row>
+    <row r="299">
+      <c r="A299" t="n">
+        <v>298</v>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>一分机场</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>https://xn--4gqx1hgtfdmt.com/#/register?code=0mMeKM0b</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr"/>
+      <c r="H299" t="inlineStr"/>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr"/>
+    </row>
+    <row r="300">
+      <c r="A300" t="n">
+        <v>299</v>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>大飞云</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>https://www.dafeixx.com/#/login?code=kRT0eCbc</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr"/>
+      <c r="H300" t="inlineStr"/>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr"/>
+    </row>
+    <row r="301">
+      <c r="A301" t="n">
+        <v>300</v>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>流量光机场</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>https://llg01.com/#/register?code=jBlwQDRb</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr"/>
+      <c r="H301" t="inlineStr"/>
+      <c r="I301" t="inlineStr"/>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>最低6.67元/月 60.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="n">
+        <v>301</v>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>北海网络</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>https://beihaiwangluo.ink/#/register?code=sPhmM6Dw</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr"/>
+      <c r="H302" t="inlineStr"/>
+      <c r="I302" t="inlineStr"/>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>最低15.83元/月 200.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="n">
+        <v>302</v>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>樱桃云 Cherry Network</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>https://board.cherrynet.work/#/register?code=XwXy9MzA</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr"/>
+      <c r="H303" t="inlineStr"/>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>接口返回错误: {'status': 'fail', 'message': '邮箱验证码有误', 'data': N</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr"/>
+    </row>
+    <row r="304">
+      <c r="A304" t="n">
+        <v>303</v>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>火麒麟</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/969.html</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr"/>
+      <c r="H304" t="inlineStr"/>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr"/>
+    </row>
+    <row r="305">
+      <c r="A305" t="n">
+        <v>304</v>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>FilmCloud</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>https://okk.filmtoday.xyz/#/register?code=yef6BgFx</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr"/>
+      <c r="H305" t="inlineStr"/>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr"/>
+    </row>
+    <row r="306">
+      <c r="A306" t="n">
+        <v>305</v>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>大坤场</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/962.html</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr"/>
+      <c r="H306" t="inlineStr"/>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" t="n">
+        <v>306</v>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>UCSS</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>https://my.undercurrentss.com/index.php?rp=/store/ucss</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr"/>
+      <c r="H307" t="inlineStr"/>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr"/>
+    </row>
+    <row r="308">
+      <c r="A308" t="n">
+        <v>307</v>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>咸鱼加速器</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>https://nexuscloud.ch/aff.php?aff=120</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr"/>
+      <c r="H308" t="inlineStr"/>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr"/>
+    </row>
+    <row r="309">
+      <c r="A309" t="n">
+        <v>308</v>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>XXAI 机场</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>http://dash.xxai.cloud/auth/register?c=pP1t059C</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr"/>
+      <c r="H309" t="inlineStr"/>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr"/>
+    </row>
+    <row r="310">
+      <c r="A310" t="n">
+        <v>309</v>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>TKV Network</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>https://portal.tkv.one/aff.php?aff=49</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr"/>
+      <c r="H310" t="inlineStr"/>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr"/>
+    </row>
+    <row r="311">
+      <c r="A311" t="n">
+        <v>310</v>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>xgCloud</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>https://www.xgyuming.com/#/register?code=mGn8DTdx</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr"/>
+      <c r="H311" t="inlineStr"/>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr"/>
+    </row>
+    <row r="312">
+      <c r="A312" t="n">
+        <v>311</v>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>速云机场</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/912.html</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr"/>
+      <c r="H312" t="inlineStr"/>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J312" t="inlineStr"/>
+    </row>
+    <row r="313">
+      <c r="A313" t="n">
+        <v>312</v>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>SS-ID</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>https://qe.newssid.com/#/register?code=ZU1wEZPu</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr"/>
+      <c r="H313" t="inlineStr"/>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr"/>
+    </row>
+    <row r="314">
+      <c r="A314" t="n">
+        <v>313</v>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>YepFast 椰皮加速</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>https://dash.yep.top/#/auth/signup;referral=Aigb7hjz</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr"/>
+      <c r="H314" t="inlineStr"/>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr"/>
+    </row>
+    <row r="315">
+      <c r="A315" t="n">
+        <v>314</v>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>顶级机场</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>https://xn--mes358a9urctx.com/#/register?code=HYtTrTUL</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr"/>
+      <c r="H315" t="inlineStr"/>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr"/>
+    </row>
+    <row r="316">
+      <c r="A316" t="n">
+        <v>315</v>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Forest VPN</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>https://forest-cn.com/download#/register?code=qQ606gGg</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr"/>
+      <c r="H316" t="inlineStr"/>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr"/>
+    </row>
+    <row r="317">
+      <c r="A317" t="n">
+        <v>316</v>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Aladdin Net 阿拉丁网络</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>https://short.thisgourl.xyz/#/register?code=67189fa7</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr"/>
+      <c r="H317" t="inlineStr"/>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr"/>
+    </row>
+    <row r="318">
+      <c r="A318" t="n">
+        <v>317</v>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>CloudFox 云狐</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>https://cldfoxgroup.xyz/register?code=V1QTMqFv</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr"/>
+      <c r="H318" t="inlineStr"/>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr"/>
+    </row>
+    <row r="319">
+      <c r="A319" t="n">
+        <v>318</v>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>CoCo Duck 小黄鸭机场</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>https://dash.cocoduck.live/auth/register?code=11196cc1b2</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr"/>
+      <c r="H319" t="inlineStr"/>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>need_tos</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr"/>
+    </row>
+    <row r="320">
+      <c r="A320" t="n">
+        <v>319</v>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>三分机场</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/850.html</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr"/>
+      <c r="H320" t="inlineStr"/>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr"/>
+    </row>
+    <row r="321">
+      <c r="A321" t="n">
+        <v>320</v>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>一元机场</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>https://xn--4gq62f52gdss.com/</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr"/>
+      <c r="H321" t="inlineStr"/>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr"/>
+    </row>
+    <row r="322">
+      <c r="A322" t="n">
+        <v>321</v>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>小鸡快跑 Chicken Run</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/842.html</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr"/>
+      <c r="H322" t="inlineStr"/>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr"/>
+    </row>
+    <row r="323">
+      <c r="A323" t="n">
+        <v>322</v>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Titan</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>https://eleme.pro/auth/register?code=xhdGvoBswf</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr"/>
+      <c r="H323" t="inlineStr"/>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J323" t="inlineStr"/>
+    </row>
+    <row r="324">
+      <c r="A324" t="n">
+        <v>323</v>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>1云梯</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>https://1ytheizi02.cc/register?aff=vgGd3wHY</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr"/>
+      <c r="H324" t="inlineStr"/>
+      <c r="I324" t="inlineStr"/>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>最低7.0元/月 60.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="n">
+        <v>324</v>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>rancho</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>https://yy.mcwy.pro#/register?code=fBsxhsuH</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr"/>
+      <c r="H325" t="inlineStr"/>
+      <c r="I325" t="inlineStr"/>
+      <c r="J325" t="inlineStr"/>
+    </row>
+    <row r="326">
+      <c r="A326" t="n">
+        <v>325</v>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>NieRCloud 尼尔云</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>https://board.cloudnier.com/#/register?code=VZPi9tX2</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr"/>
+      <c r="H326" t="inlineStr"/>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>接口返回错误: {'code': 400, 'message': '邮箱已在系统中存在', 'payload': N</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr"/>
+    </row>
+    <row r="327">
+      <c r="A327" t="n">
+        <v>326</v>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>渔舍</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>https://my.yushe.org/#/register?code=rhzFZjrW</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr"/>
+      <c r="H327" t="inlineStr"/>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr"/>
+    </row>
+    <row r="328">
+      <c r="A328" t="n">
+        <v>327</v>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>CornSS</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>https://www.corntt.com/#/register?code=lsuhgpKi</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr"/>
+      <c r="H328" t="inlineStr"/>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr"/>
+    </row>
+    <row r="329">
+      <c r="A329" t="n">
+        <v>328</v>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>疾风云</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>https://j36.net?code=f94g</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr"/>
+      <c r="H329" t="inlineStr"/>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr"/>
+    </row>
+    <row r="330">
+      <c r="A330" t="n">
+        <v>329</v>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>PP 机场</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>https://v2b.pp.st/register?code=JjQnh4Yp</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr"/>
+      <c r="H330" t="inlineStr"/>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>接口返回错误: {'type': 'https://developers.cloudflare.com/suppor</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr"/>
+    </row>
+    <row r="331">
+      <c r="A331" t="n">
+        <v>330</v>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>蓝星云</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>https://a.a0079.store/#/register?code=jI0lhTuz</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr"/>
+      <c r="H331" t="inlineStr"/>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr"/>
+    </row>
+    <row r="332">
+      <c r="A332" t="n">
+        <v>331</v>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>蓝帆云</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>https://lanfanz.cc/?code=8LGp</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr"/>
+      <c r="H332" t="inlineStr"/>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J332" t="inlineStr"/>
+    </row>
+    <row r="333">
+      <c r="A333" t="n">
+        <v>332</v>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>逐日</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/706.html</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr"/>
+      <c r="H333" t="inlineStr"/>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr"/>
+    </row>
+    <row r="334">
+      <c r="A334" t="n">
+        <v>333</v>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Cherry VPN</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>https://2026-04-15.sqllq.com/en/?chyvpn.cyou</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G334" t="inlineStr"/>
+      <c r="H334" t="inlineStr"/>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr"/>
+    </row>
+    <row r="335">
+      <c r="A335" t="n">
+        <v>334</v>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>智连云</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/686.html</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr"/>
+      <c r="H335" t="inlineStr"/>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J335" t="inlineStr"/>
+    </row>
+    <row r="336">
+      <c r="A336" t="n">
+        <v>335</v>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>ssLinks</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>https://123s.co/#/register?code=qc2azO1P</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr"/>
+      <c r="H336" t="inlineStr"/>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J336" t="inlineStr"/>
+    </row>
+    <row r="337">
+      <c r="A337" t="n">
+        <v>336</v>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>DegYax</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>https://degyax.com/user#/register?code=8sY7Vv1j</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr"/>
+      <c r="H337" t="inlineStr"/>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J337" t="inlineStr"/>
+    </row>
+    <row r="338">
+      <c r="A338" t="n">
+        <v>337</v>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>玉兔机场</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/667.html</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr"/>
+      <c r="H338" t="inlineStr"/>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J338" t="inlineStr"/>
+    </row>
+    <row r="339">
+      <c r="A339" t="n">
+        <v>338</v>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>233 Network</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/644.html</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr"/>
+      <c r="H339" t="inlineStr"/>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J339" t="inlineStr"/>
+    </row>
+    <row r="340">
+      <c r="A340" t="n">
+        <v>339</v>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>海獭机场</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/630.html</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr"/>
+      <c r="H340" t="inlineStr"/>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J340" t="inlineStr"/>
+    </row>
+    <row r="341">
+      <c r="A341" t="n">
+        <v>340</v>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>CyberAirport</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>https://cyberairport.net/</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr"/>
+      <c r="H341" t="inlineStr"/>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J341" t="inlineStr"/>
+    </row>
+    <row r="342">
+      <c r="A342" t="n">
+        <v>341</v>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>FacMata</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/615.html</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr"/>
+      <c r="H342" t="inlineStr"/>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J342" t="inlineStr"/>
+    </row>
+    <row r="343">
+      <c r="A343" t="n">
+        <v>342</v>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>RecMata</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/614.html</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr"/>
+      <c r="H343" t="inlineStr"/>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J343" t="inlineStr"/>
+    </row>
+    <row r="344">
+      <c r="A344" t="n">
+        <v>343</v>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Nice Duck</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>https://x.niceduck.sh/register?code=385tSEHj</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr"/>
+      <c r="H344" t="inlineStr"/>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J344" t="inlineStr"/>
+    </row>
+    <row r="345">
+      <c r="A345" t="n">
+        <v>344</v>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>小鲤鱼机场</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>https://www.xiaoliyu.me/#/register?code=90tauz2G</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr"/>
+      <c r="H345" t="inlineStr"/>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J345" t="inlineStr"/>
+    </row>
+    <row r="346">
+      <c r="A346" t="n">
+        <v>345</v>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>DuckGOGO</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>https://b.duckgogo.net/signup?code=J1KNY2W7</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr"/>
+      <c r="H346" t="inlineStr"/>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J346" t="inlineStr"/>
+    </row>
+    <row r="347">
+      <c r="A347" t="n">
+        <v>346</v>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>NO626｜游乐园</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/567.html</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr"/>
+      <c r="H347" t="inlineStr"/>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J347" t="inlineStr"/>
+    </row>
+    <row r="348">
+      <c r="A348" t="n">
+        <v>347</v>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Echo Network</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>https://echonetwork.club/#/register?code=J55pOFO9</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr"/>
+      <c r="H348" t="inlineStr"/>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J348" t="inlineStr"/>
+    </row>
+    <row r="349">
+      <c r="A349" t="n">
+        <v>348</v>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>最萌的云</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>https://www.cutecloud.net/register?code=qJWl8mot</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr"/>
+      <c r="H349" t="inlineStr"/>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J349" t="inlineStr"/>
+    </row>
+    <row r="350">
+      <c r="A350" t="n">
+        <v>349</v>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>百变小樱</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>https://bbxy.xn--cesw6hd3s99f.com/auth/register?code=lTDA</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr"/>
+      <c r="H350" t="inlineStr"/>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J350" t="inlineStr"/>
+    </row>
+    <row r="351">
+      <c r="A351" t="n">
+        <v>350</v>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>OKANC</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>https://www.okads.top?path=register&amp;code=dtSA4q3S</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr"/>
+      <c r="H351" t="inlineStr"/>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J351" t="inlineStr"/>
+    </row>
+    <row r="352">
+      <c r="A352" t="n">
+        <v>351</v>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Ten Cloud 腾云机场</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>https://cn.tencloud.net/#/register?code=uOqsMIHE</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr"/>
+      <c r="H352" t="inlineStr"/>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>接口返回错误: {'error': {'code': '404', 'message': 'The page cou</t>
+        </is>
+      </c>
+      <c r="J352" t="inlineStr"/>
+    </row>
+    <row r="353">
+      <c r="A353" t="n">
+        <v>352</v>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>拿铁云 Latte Cloud</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>https://natieyun.men/#/register?code=Q2pYpBYm</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr"/>
+      <c r="H353" t="inlineStr"/>
+      <c r="I353" t="inlineStr"/>
+      <c r="J353" t="inlineStr">
+        <is>
+          <t>最低16.67元/月 400.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="n">
+        <v>353</v>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>FSCloud</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>https://web.fscloud.cc/#/register?code=o8HSLd25</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr"/>
+      <c r="H354" t="inlineStr"/>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J354" t="inlineStr"/>
+    </row>
+    <row r="355">
+      <c r="A355" t="n">
+        <v>354</v>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>NessByte 耐思云</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>https://zone3.nessbyte.top/#/register?code=TbFaOU54</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr"/>
+      <c r="H355" t="inlineStr"/>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J355" t="inlineStr"/>
+    </row>
+    <row r="356">
+      <c r="A356" t="n">
+        <v>355</v>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>八戒机场</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>https://bajie.pw/#/register?code=tEtqE2HX</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>注册失败-发验证码失败</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr"/>
+      <c r="H356" t="inlineStr"/>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>请求发送验证码接口失败/被拦截</t>
+        </is>
+      </c>
+      <c r="J356" t="inlineStr"/>
+    </row>
+    <row r="357">
+      <c r="A357" t="n">
+        <v>356</v>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>ESNC 东急</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>https://esnc.link/#/register?code=YXd2NPEU</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr"/>
+      <c r="H357" t="inlineStr"/>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J357" t="inlineStr"/>
+    </row>
+    <row r="358">
+      <c r="A358" t="n">
+        <v>357</v>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Dual Net</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>https://client.neodualnet.com/#/register?code=Qpua8rG9</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>注册失败-发验证码失败</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr"/>
+      <c r="H358" t="inlineStr"/>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>请求发送验证码接口失败/被拦截</t>
+        </is>
+      </c>
+      <c r="J358" t="inlineStr"/>
+    </row>
+    <row r="359">
+      <c r="A359" t="n">
+        <v>358</v>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>辉夜 Proxy</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>https://user.hyproxy.cc/#/register?code=1fd33Yx9</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>注册失败-发验证码失败</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr"/>
+      <c r="H359" t="inlineStr"/>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>请求发送验证码接口失败/被拦截</t>
+        </is>
+      </c>
+      <c r="J359" t="inlineStr"/>
+    </row>
+    <row r="360">
+      <c r="A360" t="n">
+        <v>359</v>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Helium Network 氦网</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>https://web.henet.uk/#/register?code=4fIEpyGj</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>注册失败-发验证码失败</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr"/>
+      <c r="H360" t="inlineStr"/>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>请求发送验证码接口失败/被拦截</t>
+        </is>
+      </c>
+      <c r="J360" t="inlineStr"/>
+    </row>
+    <row r="361">
+      <c r="A361" t="n">
+        <v>360</v>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>OK Cloud</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/313.html</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr"/>
+      <c r="H361" t="inlineStr"/>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J361" t="inlineStr"/>
+    </row>
+    <row r="362">
+      <c r="A362" t="n">
+        <v>361</v>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Starnet</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>https://www.starnetcn.com/#/register?code=Tah9e1Tk</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr"/>
+      <c r="H362" t="inlineStr"/>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J362" t="inlineStr"/>
+    </row>
+    <row r="363">
+      <c r="A363" t="n">
+        <v>362</v>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Shinkansen</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/276.html</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr"/>
+      <c r="H363" t="inlineStr"/>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J363" t="inlineStr"/>
+    </row>
+    <row r="364">
+      <c r="A364" t="n">
+        <v>363</v>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>极客云</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>https://jike467.xyz/auth/register?code=bOTU</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr"/>
+      <c r="H364" t="inlineStr"/>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J364" t="inlineStr"/>
+    </row>
+    <row r="365">
+      <c r="A365" t="n">
+        <v>364</v>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>蛋挞云</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>https://eggtart.cloud/zh/#/auth/signup;referral=bx9GEfgf</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr"/>
+      <c r="H365" t="inlineStr"/>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J365" t="inlineStr"/>
+    </row>
+    <row r="366">
+      <c r="A366" t="n">
+        <v>365</v>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>OuO Network</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>https://dash.ouonetwork.com/WAF/VERIFY/CAPTCHA?info=tzk3Z9CE8hlIOICwa5RuigZd3SVUfqkajVhgBJevLxkxj8BXufxuCq30Dsk6ZWC9eRf6MbMdFijRhrh%2BTeKfJAPtlkPYpu6BZJZn4ho8gBQkdjI%3D&amp;from=%2Fregister%3Fi%3DjYwTjfHk</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr"/>
+      <c r="H366" t="inlineStr"/>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J366" t="inlineStr"/>
+    </row>
+    <row r="367">
+      <c r="A367" t="n">
+        <v>366</v>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>NaiU 机场</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>https://1224.pork.immo/#/register?code=1DWfoJID</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr"/>
+      <c r="H367" t="inlineStr"/>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J367" t="inlineStr"/>
+    </row>
+    <row r="368">
+      <c r="A368" t="n">
+        <v>367</v>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>飞兔云</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>https://301.xn--h5qy75o.vip/index.html?register=XgHqM8he</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr"/>
+      <c r="H368" t="inlineStr"/>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J368" t="inlineStr"/>
+    </row>
+    <row r="369">
+      <c r="A369" t="n">
+        <v>368</v>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>收藏柜里行走的十元unu机场店</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>https://portal.ununetwork.top/#/register?code=ClnDoDlh</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr"/>
+      <c r="H369" t="inlineStr"/>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J369" t="inlineStr"/>
+    </row>
+    <row r="370">
+      <c r="A370" t="n">
+        <v>369</v>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>狗狗加速</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>https://panel.dg1.top/#/register?code=VjaIfJte</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr"/>
+      <c r="H370" t="inlineStr"/>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J370" t="inlineStr"/>
+    </row>
+    <row r="371">
+      <c r="A371" t="n">
+        <v>370</v>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>ETON</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>https://eton.club/#/register?code=GhxcjyAn</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>注册失败-发验证码失败</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr"/>
+      <c r="H371" t="inlineStr"/>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>请求发送验证码接口失败/被拦截</t>
+        </is>
+      </c>
+      <c r="J371" t="inlineStr"/>
+    </row>
+    <row r="372">
+      <c r="A372" t="n">
+        <v>371</v>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>守候网络</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>https://dash16.newsntp.net/auth/register?code=Lsgfa7Wr</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr"/>
+      <c r="H372" t="inlineStr"/>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J372" t="inlineStr"/>
+    </row>
+    <row r="373">
+      <c r="A373" t="n">
+        <v>372</v>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>速云梯</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>https://suyunti168.xyz/auth/register?code=HI4Z</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr"/>
+      <c r="H373" t="inlineStr"/>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J373" t="inlineStr"/>
+    </row>
+    <row r="374">
+      <c r="A374" t="n">
+        <v>373</v>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>魔戒机场</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>https://mojie.me/#/register?code=7QuI6HSb</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr"/>
+      <c r="H374" t="inlineStr"/>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J374" t="inlineStr"/>
+    </row>
+    <row r="375">
+      <c r="A375" t="n">
+        <v>374</v>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>飞机云</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>https://feijiyun66.com/auth/register?code=GitR</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr"/>
+      <c r="H375" t="inlineStr"/>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J375" t="inlineStr"/>
+    </row>
+    <row r="376">
+      <c r="A376" t="n">
+        <v>375</v>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>泡泡狗</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>https://iepl.io/#/register?code=EDun6zhT</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>跳过-需要人机验证</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr"/>
+      <c r="H376" t="inlineStr"/>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>检测到图形验证码或防刷系统</t>
+        </is>
+      </c>
+      <c r="J376" t="inlineStr"/>
+    </row>
+    <row r="377">
+      <c r="A377" t="n">
+        <v>376</v>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>TaiShan Net</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>https://jp.taishan.pro/register?code=qrwnIR0M</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr"/>
+      <c r="H377" t="inlineStr"/>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J377" t="inlineStr"/>
+    </row>
+    <row r="378">
+      <c r="A378" t="n">
+        <v>377</v>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>夜煞云</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>https://1.yeshayun.com/#/register&amp;code=XzzueOpB</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr"/>
+      <c r="H378" t="inlineStr"/>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J378" t="inlineStr"/>
+    </row>
+    <row r="379">
+      <c r="A379" t="n">
+        <v>378</v>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Coo Network</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>https://web.coo.wiki/#/register?code=ncAe5Jel</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr"/>
+      <c r="H379" t="inlineStr"/>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>接口返回错误: {'message': '邮箱验证码有误'}</t>
+        </is>
+      </c>
+      <c r="J379" t="inlineStr"/>
+    </row>
+    <row r="380">
+      <c r="A380" t="n">
+        <v>379</v>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>SSRDOG 机场</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>https://guatizi.com/sites/46.html</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr"/>
+      <c r="H380" t="inlineStr"/>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J380" t="inlineStr"/>
+    </row>
+    <row r="381">
+      <c r="A381" t="n">
+        <v>380</v>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Kuromis 库洛米机场</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>https://www.kurqq9.com/register?affiliate_code=f5hbCxOkx4J2E81zwMVLV</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr"/>
+      <c r="H381" t="inlineStr"/>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J381" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix: Unified node extraction function and resolved silent failure bug
</commit_message>
<xml_diff>
--- a/注册结果.xlsx
+++ b/注册结果.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,16 +470,16 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>WgetCloud 全球加速</t>
+          <t>Nexitally 奶昔机场</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://b8cfff2a4jquxdbmwbaj.wgetcloud.org/register?code=kSIN</t>
+          <t>https://nxonearth.com/?PartnerCode=dff3c6d9014f4103a09a0be914cf1aa0</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -489,7 +489,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>fisken62fd3a@ghi.hush2u.com</t>
+          <t>kalie62fdeb@5j.shopsprint.org</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -505,6 +505,166 @@
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>WgetCloud 全球加速</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://b8cfff2a4jquxdbmwbaj.wgetcloud.org/register?code=kSIN</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ilyssa62fdec@yx.hush2u.com</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MESL Cloud</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://dc.makemesl.com/#/register?code=4NeduiXM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>moritz62fdec@21.cloudvxz.com</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>FlowerCloud 花云</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://api-flowercloud.com/aff.php?aff=17304</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>libbie62fdec@tz.accesswiki.net</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Viking Links</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://feeds.viking-links.tech/#/login?code=MaFTn476</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>https://pics9.sknil-gnikiv.com/wx5TqEUTwXks/v1/w7LQhnaSTnjD/VikingLinks?token=748dcb17331d3175ffab97ae65b2e4b4.214elsz6dkr.jpg</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>pics9.sknil-gnikiv.com</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>最低27.5元/月 250.0GB</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Auto-buy free plans to activate subscription nodes
</commit_message>
<xml_diff>
--- a/注册结果.xlsx
+++ b/注册结果.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,16 +470,16 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>千速喵</t>
+          <t>NanoPort</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://training.lilt-pupu.cc/#/register?code=3C7AZ91U</t>
+          <t>https://xn--i8s3q176n.xyz/#/register?code=RUWOjGEr</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -489,7 +489,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>goldie62fe75@zh.hush2u.com</t>
+          <t>baillie635aaa@2b.hush2u.com</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -508,26 +508,26 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NanoPort</t>
+          <t>平价机场</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://xn--i8s3q176n.xyz/#/register?code=RUWOjGEr</t>
+          <t>https://xn--6nq44rp7f3wj.com/#/register?code=KhBrweRx</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>跳过-Cloudflare</t>
+          <t>注册失败-发验证码失败</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>v9nvefwgv3@ruutukf.com</t>
+          <t>moneyflysubssr@gmail.com</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -539,33 +539,33 @@
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Cloudflare 防护</t>
+          <t>请求发送验证码接口失败/被拦截</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BYTEDOG 字节狗</t>
+          <t>Mitce</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://gate.bytedog.icu/#/register?code=Achy5PZ1</t>
+          <t>http://mitce.net</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>注册失败-发验证码失败</t>
+          <t>跳过-Cloudflare</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>x2pmwgo3vi@yzcalo.com</t>
+          <t>brittne635aab@7d.accesswiki.net</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -577,23 +577,23 @@
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>请求发送验证码接口失败/被拦截</t>
+          <t>Cloudflare 防护</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>红杏云机场</t>
+          <t>Kitty Network 机场</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://hongxingdl.com/web/#/login?code=yjburi7r</t>
+          <t>https://kitty.fo#/register?code=V5U3Hif6</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -603,7 +603,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>jkd4a8wnyo@deltajohnsons.com</t>
+          <t>schmidt635aaa@gf.sixthirtydance.org</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -622,26 +622,26 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>老头VPN</t>
+          <t>千速喵</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.chattous.net/#/register?code=LTZos9uS</t>
+          <t>https://training.lilt-pupu.cc/#/register?code=3C7AZ91U</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>跳过-无API</t>
+          <t>跳过-Cloudflare</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>sheline62fe73@1yf.cloudvxz.com</t>
+          <t>andreana635aac@qcl.sixthirtydance.org</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -653,33 +653,33 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>未找到可用API端点</t>
+          <t>Cloudflare 防护</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Mitce</t>
+          <t>ASH 微斯人</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>http://mitce.net</t>
+          <t>https://app.ashcloud.io/#/register?code=ApZN2B8O</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>跳过-Cloudflare</t>
+          <t>跳过-无API</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5mfzdfu2rb@xkxkud.com</t>
+          <t>seigel635aaa@sv.cloudvxz.com</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -691,33 +691,33 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Cloudflare 防护</t>
+          <t>未找到可用API端点</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Freecat 🐾自由猫</t>
+          <t>TIRN 机场</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://us.freecat.cloud/register?code=egkOebRs</t>
+          <t>https://tirn.top/#/register?code=bCGNZFdG</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>跳过-无API</t>
+          <t>已注册-登录成功</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>lakin62fe77@a9.sixthirtydance.org</t>
+          <t>moneyflysubssr@gmail.com</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -727,35 +727,31 @@
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>未找到可用API端点</t>
-        </is>
-      </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>UNi 独角兽机场</t>
+          <t>PixiCat</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://unis16.cc/#/register?code=tEdmBOtr</t>
+          <t>https://my.pixicat.net/register?code=mgTZN2yY</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>已注册-登录成功</t>
+          <t>跳过-无API</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>moneyflysubssr@gmail.com</t>
+          <t>adamsen635aad@kd.shopsprint.org</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -765,35 +761,35 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>最低0元/月 260.0GB</t>
-        </is>
-      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SeekNodes</t>
+          <t>狗子云</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://seeknodes.com/#/register?code=KTXoyN1q</t>
+          <t>https://dash.gzy666.top/register?code=FNHcWHjC</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>注册成功</t>
+          <t>跳过-无API</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>oi4gji9hu6@lnovic.com</t>
+          <t>arlinda635aaf@fu.accesswiki.net</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -803,31 +799,35 @@
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>冲浪猫</t>
+          <t>UNi 独角兽机场</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://guanwangdizhi.clmgo.me/#/register?code=OrjHaFhp</t>
+          <t>https://unis16.cc/#/register?code=tEdmBOtr</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>跳过-无API</t>
+          <t>已注册-登录成功</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>sumner62fe7a@l4.sixthirtydance.org</t>
+          <t>moneyflysubssr@gmail.com</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -837,12 +837,768 @@
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>最低0元/月 260.0GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>15</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>渔云机场</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://cloudfisher.xyz/web/#/login?code=N40ylSAJ</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ilyse635aaf@3a.cloudvxz.com</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
         <is>
           <t>未找到可用API端点</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>17</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>八云网络</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://8yun.me/#/register?code=CXTZu2fC</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>跳过-关闭注册</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>站点已关闭注册</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>19</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SsdAirport</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://bangpi.top?path=register&amp;code=p1HsQa0W</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>blodgett635ab3@naj.shopsprint.org</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>冲上云霄</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://9.999865.xyz/?r=21769</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>heilner635aaf@an.sixthirtydance.org</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>18</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Bocchi</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://xb.bocchi.ooo/#/register?code=4skRa5AQ</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>cuthburt635ab3@54k.hush2u.com</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>云通机场</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://yuntong.one/#/?code=4V6nzPVf</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>amandy635ab3@xz.cloudvxz.com</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>9</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Nyxen 机场</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://nyxen.org/WAF/VERIFY/CAPTCHA?info=7ogvKgNhbhq4603kX8qfjfMq%2FA2qWAp9E%2F7YVclghPi%2FSZwRUzv5uF4Bvdk3dNUtNh545Cnis6QnUyxwS6EkdjI%3D&amp;from=%2F#/register?code=t7Tca0WJ</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>10</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>柠檬宝机场 VPN</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://wws.xn--pbt38zg4v.com/#/register?code=e5Zuc4pA</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>接口返回错误: {'status': 'fail', 'message': '邮箱验证码有误', 'data': N</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>23</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>蜂窝加速器</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://h.fengwo.online/#/login?code=bbAilrMO</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>注册失败-发验证码失败</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>rooney635ab5@3h.cloudvxz.com</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>请求发送验证码接口失败/被拦截</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>26</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>独角兽机场</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://91unicorn.cloud/#/register?code=QjfbQ0DD</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>跳过-Cloudflare</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>bibi635ab7@ag.cloudvxz.com</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Cloudflare 防护</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>2</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SeekNodes</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://seeknodes.com/#/register?code=KTXoyN1q</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>cannon635aab@ndk.tohal.org</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>接口返回错误: {'message': '邮箱验证码有误'}</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>25</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>尔湾云</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://erwan.cc/auth/register?code=Lp8Mst</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>joleen635ab6@6s.sixthirtydance.org</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>24</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>PK Cloud 皮卡丘机场</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://pkhub.net/#/login?code=OuCU7jw4</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>已注册-登录成功</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>28</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>小旋风机场</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://a04.xxfvipaff.pro/#/register?inviteCode=FFA946C92AE8</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>loren635ab8@4aj.cloudvxz.com</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>30</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>特价机场</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://82af8b68-c1c0-4897-af7e-bddf32c69b2f.75733.xyz/#/register?code=ABH5upjf</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>注册失败-发验证码失败</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>请求发送验证码接口失败/被拦截</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>27</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>红岸加速</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://hongango.vip#/register?code=6yzVxr0l</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>clarabelle635ab8@46j.sixthirtydance.org</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>29</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>BigME 大米加速</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://1s.bigmeok.me/user#/register?code=WqCa8IRh</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>abagail635ab9@ymj.cloudvxz.com</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>21</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>柚子兔网络</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://yzt.moe/#/register?code=ktDtwtiD</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>注册失败</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>接口返回错误: {'message': '邮箱验证码有误'}</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>22</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>五树云</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://xiaomiaff.pro/register.html?invitecode=8UctYVq0</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>跳过-不可达</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>moneyflysubssr@gmail.com</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>连接失败或超时</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>20</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>万达云</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://app.wdycenter.com/register?code=mfnTlrSw</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>跳过-无API</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>maccarone635ab6@gg.hush2u.com</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Sikeming001@</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>未找到可用API端点</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>